<commit_message>
format changes; no data changes
</commit_message>
<xml_diff>
--- a/src/technology/small-modular-reactor/conceptb-inputs.xlsx
+++ b/src/technology/small-modular-reactor/conceptb-inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\small-modular-reactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A6B23F-2523-47E7-A912-8275A84AB514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02AF5AC-2334-4E28-9126-D3079952FFF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8445" yWindow="930" windowWidth="23130" windowHeight="17685" xr2:uid="{C3FE9FA1-298D-4EB2-913D-F2BF73C3B228}"/>
+    <workbookView xWindow="36210" yWindow="90" windowWidth="15405" windowHeight="20805" xr2:uid="{C3FE9FA1-298D-4EB2-913D-F2BF73C3B228}"/>
   </bookViews>
   <sheets>
     <sheet name="Costs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>Account</t>
   </si>
@@ -184,9 +184,6 @@
   </si>
   <si>
     <t>Interest</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>60s - Subtotal</t>
@@ -1180,11 +1177,8 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="B51" t="s">
         <v>49</v>
-      </c>
-      <c r="B51" t="s">
-        <v>50</v>
       </c>
       <c r="C51">
         <v>592300800</v>
@@ -1192,7 +1186,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C52">
         <v>1906</v>
@@ -1200,7 +1194,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C54">
         <v>1596758321</v>
@@ -1208,7 +1202,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C55">
         <v>5138</v>
@@ -1216,7 +1210,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C57">
         <v>2408936272</v>
@@ -1224,7 +1218,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C58">
         <v>7751</v>
@@ -1232,7 +1226,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C60">
         <v>2437538300</v>
@@ -1240,7 +1234,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C61">
         <v>7843</v>
@@ -1248,7 +1242,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C63">
         <v>3029839099</v>
@@ -1256,7 +1250,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C64">
         <v>9749</v>
@@ -1264,7 +1258,7 @@
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C66">
         <v>2437538300</v>
@@ -1272,7 +1266,7 @@
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C67">
         <v>7843</v>
@@ -1280,7 +1274,7 @@
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C69">
         <v>3029839099</v>
@@ -1288,7 +1282,7 @@
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C70">
         <v>9749</v>
@@ -1306,16 +1300,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>65</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>66</v>
-      </c>
-      <c r="D1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>